<commit_message>
Add 14 India healthcare publications; fix direct-feed RSS discovery
Adds 14 India-focused sources (entries #34–47) to the "Newsletters &
Publications" tab of inputs/voices.xlsx: Entrackr, Medical Dialogues,
Digital Health News, Business Standard (Health & IPO), MediaNama, BioVoice
News, IndiaMedToday, eHealth Magazine, Life Science India, Express Pharma,
The Ken (Healthcare), PIB Press Releases, and Fortune India.

Several of these are configured with direct feed URLs (.rss / .xml / /feed).
The feed-discovery logic only tried heuristic path appends (/feed, /rss, …)
and an HTML <link rel="alternate"> fallback — it never checked whether the
configured URL was itself a feed, so valid direct-feed URLs yielded zero
items. _discover_with_body (and its async twin) now use the URL as-is when it
parses as a feed (discovery="direct"), reusing the fallback GET so there is no
extra request. Adds unit + end-to-end tests.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inputs/voices.xlsx
+++ b/inputs/voices.xlsx
@@ -167,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -228,6 +228,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16498,7 +16504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H35"/>
+  <dimension ref="A2:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.75"/>
   <cols>
     <col width="5" customWidth="1" style="21" min="1" max="1"/>
@@ -17870,6 +17876,566 @@
       <c r="H35" s="7" t="inlineStr">
         <is>
           <t>https://www.generalist.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>Entrackr</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication / Newsletter</t>
+        </is>
+      </c>
+      <c r="E36" s="22" t="inlineStr">
+        <is>
+          <t>Bareback Media</t>
+        </is>
+      </c>
+      <c r="F36" s="22" t="inlineStr">
+        <is>
+          <t>India startup funding scoops, M&amp;A, IPO/DRHP filings, monthly funding reports.</t>
+        </is>
+      </c>
+      <c r="G36" s="22" t="inlineStr">
+        <is>
+          <t>Very high startup-ecosystem reach</t>
+        </is>
+      </c>
+      <c r="H36" s="23" t="inlineStr">
+        <is>
+          <t>https://entrackr.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="22" t="inlineStr">
+        <is>
+          <t>Medical Dialogues</t>
+        </is>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication</t>
+        </is>
+      </c>
+      <c r="E37" s="22" t="inlineStr">
+        <is>
+          <t>Minerva Medical Treatment</t>
+        </is>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>NMC, CDSCO approvals &amp; bans, NPPA pricing, hospital and medico-legal news.</t>
+        </is>
+      </c>
+      <c r="G37" s="22" t="inlineStr">
+        <is>
+          <t>Very high (1M+ monthly readers)</t>
+        </is>
+      </c>
+      <c r="H37" s="23" t="inlineStr">
+        <is>
+          <t>https://medicaldialogues.in/custom_feeds.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="22" t="inlineStr">
+        <is>
+          <t>Digital Health News (DHN)</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication</t>
+        </is>
+      </c>
+      <c r="E38" s="22" t="inlineStr">
+        <is>
+          <t>DHN (Vishnu Saxena)</t>
+        </is>
+      </c>
+      <c r="F38" s="22" t="inlineStr">
+        <is>
+          <t>India digital health, ABDM, healthtech funding recaps, hospital tech.</t>
+        </is>
+      </c>
+      <c r="G38" s="22" t="inlineStr">
+        <is>
+          <t>Growing India digital-health-native reach</t>
+        </is>
+      </c>
+      <c r="H38" s="23" t="inlineStr">
+        <is>
+          <t>https://www.digitalhealthnews.com/feed</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Business Standard — Health</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Mainstream Business Media</t>
+        </is>
+      </c>
+      <c r="E39" s="22" t="inlineStr">
+        <is>
+          <t>Business Standard</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>Hospital and pharma M&amp;A, earnings, healthcare policy.</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="inlineStr">
+        <is>
+          <t>Very high</t>
+        </is>
+      </c>
+      <c r="H39" s="23" t="inlineStr">
+        <is>
+          <t>https://www.business-standard.com/rss/health-185.rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>Business Standard — IPO</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>Mainstream Business Media</t>
+        </is>
+      </c>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>Business Standard</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>IPO filings and listings incl. hospital and diagnostics chains.</t>
+        </is>
+      </c>
+      <c r="G40" s="22" t="inlineStr">
+        <is>
+          <t>Very high</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>https://www.business-standard.com/rss/markets/ipo-10611.rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
+        <is>
+          <t>MediaNama</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>Policy Publication</t>
+        </is>
+      </c>
+      <c r="E41" s="22" t="inlineStr">
+        <is>
+          <t>Mixed Bag Media (Nikhil Pahwa)</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="inlineStr">
+        <is>
+          <t>DPDP Act, health data, digital health regulation.</t>
+        </is>
+      </c>
+      <c r="G41" s="22" t="inlineStr">
+        <is>
+          <t>High policy authority</t>
+        </is>
+      </c>
+      <c r="H41" s="23" t="inlineStr">
+        <is>
+          <t>https://www.medianama.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>BioVoice News</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>BioVoice News (Rahul Koul)</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr">
+        <is>
+          <t>Biotech, biopharma, medtech, diagnostics; CDSCO approvals.</t>
+        </is>
+      </c>
+      <c r="G42" s="22" t="inlineStr">
+        <is>
+          <t>Niche but well-networked</t>
+        </is>
+      </c>
+      <c r="H42" s="23" t="inlineStr">
+        <is>
+          <t>https://biovoicenews.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>IndiaMedToday</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication</t>
+        </is>
+      </c>
+      <c r="E43" s="22" t="inlineStr">
+        <is>
+          <t>IndiaMedToday</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="inlineStr">
+        <is>
+          <t>Medtech and devices: funds, localisation, distributor and hospital deals, device policy.</t>
+        </is>
+      </c>
+      <c r="G43" s="22" t="inlineStr">
+        <is>
+          <t>Small but on-beat for devices</t>
+        </is>
+      </c>
+      <c r="H43" s="23" t="inlineStr">
+        <is>
+          <t>https://indiamedtoday.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>eHealth Magazine</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>Elets Technomedia</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>Hospital IT, ABDM, government health tech, health insurance tech.</t>
+        </is>
+      </c>
+      <c r="G44" s="22" t="inlineStr">
+        <is>
+          <t>Established govt/PSU-facing reach</t>
+        </is>
+      </c>
+      <c r="H44" s="23" t="inlineStr">
+        <is>
+          <t>https://ehealth.eletsonline.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Life Science India</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>Newsletter (Substack)</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>Independent analyst</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>Thesis-level analysis of Indian pharma and healthcare markets and investor activity.</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="inlineStr">
+        <is>
+          <t>Small but analytical</t>
+        </is>
+      </c>
+      <c r="H45" s="23" t="inlineStr">
+        <is>
+          <t>https://lifescienceindia.substack.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Express Pharma</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>Trade Publication</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>Indian Express Group</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>India pharma business, DRHP/IPO filings, CDSCO/DCGI and US FDA approvals.</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="inlineStr">
+        <is>
+          <t>Strong industry reach</t>
+        </is>
+      </c>
+      <c r="H46" s="23" t="inlineStr">
+        <is>
+          <t>https://www.expresspharma.in/feed/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>The Ken — Healthcare</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>Premium Analysis</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>Kenrise Media (Seema Singh)</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>Deep reported analysis: hospital PE roll-ups, IPOs, provider strategy. Paywalled — headlines only.</t>
+        </is>
+      </c>
+      <c r="G47" s="22" t="inlineStr">
+        <is>
+          <t>Premium and influential, ~1 story/month</t>
+        </is>
+      </c>
+      <c r="H47" s="23" t="inlineStr">
+        <is>
+          <t>https://the-ken.com/tag/healthcare/feed/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>PIB Press Releases</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>Government Wire</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>Press Information Bureau, Govt of India</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>All-ministry government releases; working proxy for MoHFW, ABDM and NPPA parent ministry. Keep reg=1 or the feed returns empty.</t>
+        </is>
+      </c>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>Authoritative primary source</t>
+        </is>
+      </c>
+      <c r="H48" s="23" t="inlineStr">
+        <is>
+          <t>https://pib.gov.in/RssMain.aspx?ModId=6&amp;Lang=1&amp;Regid=1&amp;reg=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Fortune India</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>Mainstream Business Media</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>Fortune India</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>Healthcare deals and features: provider M&amp;A, health insurance, healthtech.</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H49" s="23" t="inlineStr">
+        <is>
+          <t>https://www.fortuneindia.com/feed</t>
         </is>
       </c>
     </row>

</xml_diff>